<commit_message>
Implemented Vitamin D level of a patient into the recommender logic
</commit_message>
<xml_diff>
--- a/clean_pcos_data.xlsx
+++ b/clean_pcos_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V469"/>
+  <dimension ref="A1:W469"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -527,6 +527,11 @@
           <t>Skin_Darkening_Acanthosis</t>
         </is>
       </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>Vitamin_D_ng_mL</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -595,6 +600,9 @@
       <c r="V2" t="n">
         <v>0</v>
       </c>
+      <c r="W2" t="n">
+        <v>46.3</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -663,6 +671,9 @@
       <c r="V3" t="n">
         <v>1</v>
       </c>
+      <c r="W3" t="n">
+        <v>24.8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -731,6 +742,9 @@
       <c r="V4" t="n">
         <v>0</v>
       </c>
+      <c r="W4" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -799,6 +813,9 @@
       <c r="V5" t="n">
         <v>0</v>
       </c>
+      <c r="W5" t="n">
+        <v>18.9</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -867,6 +884,9 @@
       <c r="V6" t="n">
         <v>0</v>
       </c>
+      <c r="W6" t="n">
+        <v>46.4</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -935,6 +955,9 @@
       <c r="V7" t="n">
         <v>0</v>
       </c>
+      <c r="W7" t="n">
+        <v>32.9</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1003,6 +1026,9 @@
       <c r="V8" t="n">
         <v>1</v>
       </c>
+      <c r="W8" t="n">
+        <v>19.5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1071,6 +1097,9 @@
       <c r="V9" t="n">
         <v>0</v>
       </c>
+      <c r="W9" t="n">
+        <v>29.8</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1139,6 +1168,9 @@
       <c r="V10" t="n">
         <v>0</v>
       </c>
+      <c r="W10" t="n">
+        <v>31.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1207,6 +1239,9 @@
       <c r="V11" t="n">
         <v>0</v>
       </c>
+      <c r="W11" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1275,6 +1310,9 @@
       <c r="V12" t="n">
         <v>1</v>
       </c>
+      <c r="W12" t="n">
+        <v>27.7</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1343,6 +1381,9 @@
       <c r="V13" t="n">
         <v>0</v>
       </c>
+      <c r="W13" t="n">
+        <v>29.4</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1411,6 +1452,9 @@
       <c r="V14" t="n">
         <v>0</v>
       </c>
+      <c r="W14" t="n">
+        <v>20.3</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1479,6 +1523,9 @@
       <c r="V15" t="n">
         <v>0</v>
       </c>
+      <c r="W15" t="n">
+        <v>20.4</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1547,6 +1594,9 @@
       <c r="V16" t="n">
         <v>0</v>
       </c>
+      <c r="W16" t="n">
+        <v>42.5</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1615,6 +1665,9 @@
       <c r="V17" t="n">
         <v>0</v>
       </c>
+      <c r="W17" t="n">
+        <v>11.9</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1683,6 +1736,9 @@
       <c r="V18" t="n">
         <v>0</v>
       </c>
+      <c r="W18" t="n">
+        <v>17.9</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1751,6 +1807,9 @@
       <c r="V19" t="n">
         <v>0</v>
       </c>
+      <c r="W19" t="n">
+        <v>30.1</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1819,6 +1878,9 @@
       <c r="V20" t="n">
         <v>0</v>
       </c>
+      <c r="W20" t="n">
+        <v>15.7</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1887,6 +1949,9 @@
       <c r="V21" t="n">
         <v>0</v>
       </c>
+      <c r="W21" t="n">
+        <v>24.2</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1955,6 +2020,9 @@
       <c r="V22" t="n">
         <v>1</v>
       </c>
+      <c r="W22" t="n">
+        <v>25.2</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -2023,6 +2091,9 @@
       <c r="V23" t="n">
         <v>1</v>
       </c>
+      <c r="W23" t="n">
+        <v>38.7</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -2091,6 +2162,9 @@
       <c r="V24" t="n">
         <v>0</v>
       </c>
+      <c r="W24" t="n">
+        <v>18.2</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -2159,6 +2233,9 @@
       <c r="V25" t="n">
         <v>1</v>
       </c>
+      <c r="W25" t="n">
+        <v>24.3</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2227,6 +2304,9 @@
       <c r="V26" t="n">
         <v>0</v>
       </c>
+      <c r="W26" t="n">
+        <v>14.2</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -2295,6 +2375,9 @@
       <c r="V27" t="n">
         <v>1</v>
       </c>
+      <c r="W27" t="n">
+        <v>37.1</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -2363,6 +2446,9 @@
       <c r="V28" t="n">
         <v>0</v>
       </c>
+      <c r="W28" t="n">
+        <v>32</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2431,6 +2517,9 @@
       <c r="V29" t="n">
         <v>0</v>
       </c>
+      <c r="W29" t="n">
+        <v>24.8</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2499,6 +2588,9 @@
       <c r="V30" t="n">
         <v>0</v>
       </c>
+      <c r="W30" t="n">
+        <v>18.9</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2567,6 +2659,9 @@
       <c r="V31" t="n">
         <v>0</v>
       </c>
+      <c r="W31" t="n">
+        <v>15.8</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2635,6 +2730,9 @@
       <c r="V32" t="n">
         <v>1</v>
       </c>
+      <c r="W32" t="n">
+        <v>23.3</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2703,6 +2801,9 @@
       <c r="V33" t="n">
         <v>0</v>
       </c>
+      <c r="W33" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2771,6 +2872,9 @@
       <c r="V34" t="n">
         <v>0</v>
       </c>
+      <c r="W34" t="n">
+        <v>32.2</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2839,6 +2943,9 @@
       <c r="V35" t="n">
         <v>0</v>
       </c>
+      <c r="W35" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2907,6 +3014,9 @@
       <c r="V36" t="n">
         <v>1</v>
       </c>
+      <c r="W36" t="n">
+        <v>13.6</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2975,6 +3085,9 @@
       <c r="V37" t="n">
         <v>0</v>
       </c>
+      <c r="W37" t="n">
+        <v>29.4</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -3043,6 +3156,9 @@
       <c r="V38" t="n">
         <v>1</v>
       </c>
+      <c r="W38" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -3111,6 +3227,9 @@
       <c r="V39" t="n">
         <v>1</v>
       </c>
+      <c r="W39" t="n">
+        <v>11.9</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -3179,6 +3298,9 @@
       <c r="V40" t="n">
         <v>0</v>
       </c>
+      <c r="W40" t="n">
+        <v>11.5</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -3247,6 +3369,9 @@
       <c r="V41" t="n">
         <v>0</v>
       </c>
+      <c r="W41" t="n">
+        <v>27.5</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -3315,6 +3440,9 @@
       <c r="V42" t="n">
         <v>0</v>
       </c>
+      <c r="W42" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -3383,6 +3511,9 @@
       <c r="V43" t="n">
         <v>0</v>
       </c>
+      <c r="W43" t="n">
+        <v>47.2</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -3451,6 +3582,9 @@
       <c r="V44" t="n">
         <v>1</v>
       </c>
+      <c r="W44" t="n">
+        <v>38.9</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -3519,6 +3653,9 @@
       <c r="V45" t="n">
         <v>0</v>
       </c>
+      <c r="W45" t="n">
+        <v>31.7</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -3587,6 +3724,9 @@
       <c r="V46" t="n">
         <v>0</v>
       </c>
+      <c r="W46" t="n">
+        <v>37.8</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -3655,6 +3795,9 @@
       <c r="V47" t="n">
         <v>0</v>
       </c>
+      <c r="W47" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -3723,6 +3866,9 @@
       <c r="V48" t="n">
         <v>1</v>
       </c>
+      <c r="W48" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -3791,6 +3937,9 @@
       <c r="V49" t="n">
         <v>0</v>
       </c>
+      <c r="W49" t="n">
+        <v>32.7</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -3859,6 +4008,9 @@
       <c r="V50" t="n">
         <v>0</v>
       </c>
+      <c r="W50" t="n">
+        <v>35.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -3927,6 +4079,9 @@
       <c r="V51" t="n">
         <v>0</v>
       </c>
+      <c r="W51" t="n">
+        <v>23.1</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -3995,6 +4150,9 @@
       <c r="V52" t="n">
         <v>0</v>
       </c>
+      <c r="W52" t="n">
+        <v>35.6</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -4063,6 +4221,9 @@
       <c r="V53" t="n">
         <v>1</v>
       </c>
+      <c r="W53" t="n">
+        <v>37.8</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -4131,6 +4292,9 @@
       <c r="V54" t="n">
         <v>0</v>
       </c>
+      <c r="W54" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -4199,6 +4363,9 @@
       <c r="V55" t="n">
         <v>1</v>
       </c>
+      <c r="W55" t="n">
+        <v>27.9</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -4267,6 +4434,9 @@
       <c r="V56" t="n">
         <v>0</v>
       </c>
+      <c r="W56" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -4335,6 +4505,9 @@
       <c r="V57" t="n">
         <v>1</v>
       </c>
+      <c r="W57" t="n">
+        <v>19.2</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -4403,6 +4576,9 @@
       <c r="V58" t="n">
         <v>0</v>
       </c>
+      <c r="W58" t="n">
+        <v>35.3</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -4471,6 +4647,9 @@
       <c r="V59" t="n">
         <v>1</v>
       </c>
+      <c r="W59" t="n">
+        <v>33.1</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -4539,6 +4718,9 @@
       <c r="V60" t="n">
         <v>1</v>
       </c>
+      <c r="W60" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -4607,6 +4789,9 @@
       <c r="V61" t="n">
         <v>1</v>
       </c>
+      <c r="W61" t="n">
+        <v>18.5</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -4675,6 +4860,9 @@
       <c r="V62" t="n">
         <v>0</v>
       </c>
+      <c r="W62" t="n">
+        <v>26.9</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -4743,6 +4931,9 @@
       <c r="V63" t="n">
         <v>0</v>
       </c>
+      <c r="W63" t="n">
+        <v>14.9</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -4811,6 +5002,9 @@
       <c r="V64" t="n">
         <v>0</v>
       </c>
+      <c r="W64" t="n">
+        <v>30.8</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -4879,6 +5073,9 @@
       <c r="V65" t="n">
         <v>0</v>
       </c>
+      <c r="W65" t="n">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -4947,6 +5144,9 @@
       <c r="V66" t="n">
         <v>1</v>
       </c>
+      <c r="W66" t="n">
+        <v>19.5</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -5015,6 +5215,9 @@
       <c r="V67" t="n">
         <v>0</v>
       </c>
+      <c r="W67" t="n">
+        <v>27.6</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -5083,6 +5286,9 @@
       <c r="V68" t="n">
         <v>1</v>
       </c>
+      <c r="W68" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -5151,6 +5357,9 @@
       <c r="V69" t="n">
         <v>0</v>
       </c>
+      <c r="W69" t="n">
+        <v>24.9</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -5219,6 +5428,9 @@
       <c r="V70" t="n">
         <v>0</v>
       </c>
+      <c r="W70" t="n">
+        <v>12.8</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -5287,6 +5499,9 @@
       <c r="V71" t="n">
         <v>0</v>
       </c>
+      <c r="W71" t="n">
+        <v>24.4</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -5355,6 +5570,9 @@
       <c r="V72" t="n">
         <v>1</v>
       </c>
+      <c r="W72" t="n">
+        <v>15.4</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -5423,6 +5641,9 @@
       <c r="V73" t="n">
         <v>0</v>
       </c>
+      <c r="W73" t="n">
+        <v>12.6</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -5491,6 +5712,9 @@
       <c r="V74" t="n">
         <v>1</v>
       </c>
+      <c r="W74" t="n">
+        <v>12.5</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -5559,6 +5783,9 @@
       <c r="V75" t="n">
         <v>1</v>
       </c>
+      <c r="W75" t="n">
+        <v>14.7</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -5627,6 +5854,9 @@
       <c r="V76" t="n">
         <v>0</v>
       </c>
+      <c r="W76" t="n">
+        <v>19.1</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -5695,6 +5925,9 @@
       <c r="V77" t="n">
         <v>0</v>
       </c>
+      <c r="W77" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -5763,6 +5996,9 @@
       <c r="V78" t="n">
         <v>0</v>
       </c>
+      <c r="W78" t="n">
+        <v>14.9</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -5831,6 +6067,9 @@
       <c r="V79" t="n">
         <v>1</v>
       </c>
+      <c r="W79" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -5899,6 +6138,9 @@
       <c r="V80" t="n">
         <v>0</v>
       </c>
+      <c r="W80" t="n">
+        <v>26.6</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -5967,6 +6209,9 @@
       <c r="V81" t="n">
         <v>1</v>
       </c>
+      <c r="W81" t="n">
+        <v>32.9</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -6035,6 +6280,9 @@
       <c r="V82" t="n">
         <v>0</v>
       </c>
+      <c r="W82" t="n">
+        <v>29.3</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -6103,6 +6351,9 @@
       <c r="V83" t="n">
         <v>0</v>
       </c>
+      <c r="W83" t="n">
+        <v>12.4</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -6171,6 +6422,9 @@
       <c r="V84" t="n">
         <v>0</v>
       </c>
+      <c r="W84" t="n">
+        <v>37.2</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -6239,6 +6493,9 @@
       <c r="V85" t="n">
         <v>1</v>
       </c>
+      <c r="W85" t="n">
+        <v>31.5</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -6307,6 +6564,9 @@
       <c r="V86" t="n">
         <v>0</v>
       </c>
+      <c r="W86" t="n">
+        <v>31.1</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -6375,6 +6635,9 @@
       <c r="V87" t="n">
         <v>0</v>
       </c>
+      <c r="W87" t="n">
+        <v>30.9</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -6443,6 +6706,9 @@
       <c r="V88" t="n">
         <v>1</v>
       </c>
+      <c r="W88" t="n">
+        <v>19.9</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -6511,6 +6777,9 @@
       <c r="V89" t="n">
         <v>0</v>
       </c>
+      <c r="W89" t="n">
+        <v>15.8</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -6579,6 +6848,9 @@
       <c r="V90" t="n">
         <v>0</v>
       </c>
+      <c r="W90" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -6647,6 +6919,9 @@
       <c r="V91" t="n">
         <v>0</v>
       </c>
+      <c r="W91" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -6715,6 +6990,9 @@
       <c r="V92" t="n">
         <v>0</v>
       </c>
+      <c r="W92" t="n">
+        <v>46.8</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -6783,6 +7061,9 @@
       <c r="V93" t="n">
         <v>0</v>
       </c>
+      <c r="W93" t="n">
+        <v>31.1</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -6851,6 +7132,9 @@
       <c r="V94" t="n">
         <v>0</v>
       </c>
+      <c r="W94" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -6919,6 +7203,9 @@
       <c r="V95" t="n">
         <v>0</v>
       </c>
+      <c r="W95" t="n">
+        <v>5.7</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -6987,6 +7274,9 @@
       <c r="V96" t="n">
         <v>0</v>
       </c>
+      <c r="W96" t="n">
+        <v>19.8</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -7055,6 +7345,9 @@
       <c r="V97" t="n">
         <v>1</v>
       </c>
+      <c r="W97" t="n">
+        <v>11.8</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -7123,6 +7416,9 @@
       <c r="V98" t="n">
         <v>0</v>
       </c>
+      <c r="W98" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -7191,6 +7487,9 @@
       <c r="V99" t="n">
         <v>0</v>
       </c>
+      <c r="W99" t="n">
+        <v>31.1</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -7259,6 +7558,9 @@
       <c r="V100" t="n">
         <v>1</v>
       </c>
+      <c r="W100" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -7327,6 +7629,9 @@
       <c r="V101" t="n">
         <v>0</v>
       </c>
+      <c r="W101" t="n">
+        <v>26.2</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -7395,6 +7700,9 @@
       <c r="V102" t="n">
         <v>0</v>
       </c>
+      <c r="W102" t="n">
+        <v>32.2</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -7463,6 +7771,9 @@
       <c r="V103" t="n">
         <v>0</v>
       </c>
+      <c r="W103" t="n">
+        <v>9.6</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -7531,6 +7842,9 @@
       <c r="V104" t="n">
         <v>0</v>
       </c>
+      <c r="W104" t="n">
+        <v>41.5</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -7599,6 +7913,9 @@
       <c r="V105" t="n">
         <v>0</v>
       </c>
+      <c r="W105" t="n">
+        <v>6.1</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -7667,6 +7984,9 @@
       <c r="V106" t="n">
         <v>0</v>
       </c>
+      <c r="W106" t="n">
+        <v>14.1</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -7735,6 +8055,9 @@
       <c r="V107" t="n">
         <v>0</v>
       </c>
+      <c r="W107" t="n">
+        <v>7.9</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -7803,6 +8126,9 @@
       <c r="V108" t="n">
         <v>0</v>
       </c>
+      <c r="W108" t="n">
+        <v>17.3</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -7871,6 +8197,9 @@
       <c r="V109" t="n">
         <v>0</v>
       </c>
+      <c r="W109" t="n">
+        <v>28.6</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -7939,6 +8268,9 @@
       <c r="V110" t="n">
         <v>1</v>
       </c>
+      <c r="W110" t="n">
+        <v>24.3</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -8007,6 +8339,9 @@
       <c r="V111" t="n">
         <v>1</v>
       </c>
+      <c r="W111" t="n">
+        <v>15.4</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -8075,6 +8410,9 @@
       <c r="V112" t="n">
         <v>1</v>
       </c>
+      <c r="W112" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -8143,6 +8481,9 @@
       <c r="V113" t="n">
         <v>1</v>
       </c>
+      <c r="W113" t="n">
+        <v>55.7</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -8211,6 +8552,9 @@
       <c r="V114" t="n">
         <v>0</v>
       </c>
+      <c r="W114" t="n">
+        <v>19.3</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -8279,6 +8623,9 @@
       <c r="V115" t="n">
         <v>0</v>
       </c>
+      <c r="W115" t="n">
+        <v>35.5</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -8347,6 +8694,9 @@
       <c r="V116" t="n">
         <v>0</v>
       </c>
+      <c r="W116" t="n">
+        <v>24.3</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -8415,6 +8765,9 @@
       <c r="V117" t="n">
         <v>1</v>
       </c>
+      <c r="W117" t="n">
+        <v>38.6</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -8483,6 +8836,9 @@
       <c r="V118" t="n">
         <v>1</v>
       </c>
+      <c r="W118" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -8551,6 +8907,9 @@
       <c r="V119" t="n">
         <v>0</v>
       </c>
+      <c r="W119" t="n">
+        <v>18.2</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -8619,6 +8978,9 @@
       <c r="V120" t="n">
         <v>0</v>
       </c>
+      <c r="W120" t="n">
+        <v>7.5</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -8687,6 +9049,9 @@
       <c r="V121" t="n">
         <v>0</v>
       </c>
+      <c r="W121" t="n">
+        <v>5.9</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -8755,6 +9120,9 @@
       <c r="V122" t="n">
         <v>1</v>
       </c>
+      <c r="W122" t="n">
+        <v>12.2</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -8823,6 +9191,9 @@
       <c r="V123" t="n">
         <v>0</v>
       </c>
+      <c r="W123" t="n">
+        <v>24.8</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -8891,6 +9262,9 @@
       <c r="V124" t="n">
         <v>1</v>
       </c>
+      <c r="W124" t="n">
+        <v>10.3</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -8959,6 +9333,9 @@
       <c r="V125" t="n">
         <v>0</v>
       </c>
+      <c r="W125" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -9027,6 +9404,9 @@
       <c r="V126" t="n">
         <v>1</v>
       </c>
+      <c r="W126" t="n">
+        <v>26.8</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -9095,6 +9475,9 @@
       <c r="V127" t="n">
         <v>1</v>
       </c>
+      <c r="W127" t="n">
+        <v>29.6</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -9163,6 +9546,9 @@
       <c r="V128" t="n">
         <v>0</v>
       </c>
+      <c r="W128" t="n">
+        <v>14.9</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -9231,6 +9617,9 @@
       <c r="V129" t="n">
         <v>0</v>
       </c>
+      <c r="W129" t="n">
+        <v>16.3</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -9299,6 +9688,9 @@
       <c r="V130" t="n">
         <v>0</v>
       </c>
+      <c r="W130" t="n">
+        <v>24.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -9367,6 +9759,9 @@
       <c r="V131" t="n">
         <v>0</v>
       </c>
+      <c r="W131" t="n">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -9435,6 +9830,9 @@
       <c r="V132" t="n">
         <v>1</v>
       </c>
+      <c r="W132" t="n">
+        <v>25.5</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -9503,6 +9901,9 @@
       <c r="V133" t="n">
         <v>0</v>
       </c>
+      <c r="W133" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -9571,6 +9972,9 @@
       <c r="V134" t="n">
         <v>0</v>
       </c>
+      <c r="W134" t="n">
+        <v>28.3</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -9639,6 +10043,9 @@
       <c r="V135" t="n">
         <v>0</v>
       </c>
+      <c r="W135" t="n">
+        <v>21.1</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -9707,6 +10114,9 @@
       <c r="V136" t="n">
         <v>0</v>
       </c>
+      <c r="W136" t="n">
+        <v>27.6</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -9775,6 +10185,9 @@
       <c r="V137" t="n">
         <v>0</v>
       </c>
+      <c r="W137" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -9843,6 +10256,9 @@
       <c r="V138" t="n">
         <v>0</v>
       </c>
+      <c r="W138" t="n">
+        <v>34.9</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -9911,6 +10327,9 @@
       <c r="V139" t="n">
         <v>1</v>
       </c>
+      <c r="W139" t="n">
+        <v>37.8</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -9979,6 +10398,9 @@
       <c r="V140" t="n">
         <v>0</v>
       </c>
+      <c r="W140" t="n">
+        <v>13.5</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -10047,6 +10469,9 @@
       <c r="V141" t="n">
         <v>0</v>
       </c>
+      <c r="W141" t="n">
+        <v>12.9</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -10115,6 +10540,9 @@
       <c r="V142" t="n">
         <v>0</v>
       </c>
+      <c r="W142" t="n">
+        <v>29.8</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -10183,6 +10611,9 @@
       <c r="V143" t="n">
         <v>0</v>
       </c>
+      <c r="W143" t="n">
+        <v>14.5</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -10251,6 +10682,9 @@
       <c r="V144" t="n">
         <v>0</v>
       </c>
+      <c r="W144" t="n">
+        <v>19.4</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -10319,6 +10753,9 @@
       <c r="V145" t="n">
         <v>0</v>
       </c>
+      <c r="W145" t="n">
+        <v>20.6</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -10387,6 +10824,9 @@
       <c r="V146" t="n">
         <v>1</v>
       </c>
+      <c r="W146" t="n">
+        <v>11.6</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -10455,6 +10895,9 @@
       <c r="V147" t="n">
         <v>0</v>
       </c>
+      <c r="W147" t="n">
+        <v>30.8</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -10523,6 +10966,9 @@
       <c r="V148" t="n">
         <v>0</v>
       </c>
+      <c r="W148" t="n">
+        <v>10.4</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -10591,6 +11037,9 @@
       <c r="V149" t="n">
         <v>0</v>
       </c>
+      <c r="W149" t="n">
+        <v>27.4</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -10659,6 +11108,9 @@
       <c r="V150" t="n">
         <v>0</v>
       </c>
+      <c r="W150" t="n">
+        <v>19.8</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -10727,6 +11179,9 @@
       <c r="V151" t="n">
         <v>0</v>
       </c>
+      <c r="W151" t="n">
+        <v>24.9</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -10795,6 +11250,9 @@
       <c r="V152" t="n">
         <v>1</v>
       </c>
+      <c r="W152" t="n">
+        <v>32</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -10863,6 +11321,9 @@
       <c r="V153" t="n">
         <v>1</v>
       </c>
+      <c r="W153" t="n">
+        <v>25.2</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -10931,6 +11392,9 @@
       <c r="V154" t="n">
         <v>1</v>
       </c>
+      <c r="W154" t="n">
+        <v>38.4</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -10999,6 +11463,9 @@
       <c r="V155" t="n">
         <v>0</v>
       </c>
+      <c r="W155" t="n">
+        <v>27.9</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -11067,6 +11534,9 @@
       <c r="V156" t="n">
         <v>0</v>
       </c>
+      <c r="W156" t="n">
+        <v>29.5</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -11135,6 +11605,9 @@
       <c r="V157" t="n">
         <v>1</v>
       </c>
+      <c r="W157" t="n">
+        <v>25.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -11203,6 +11676,9 @@
       <c r="V158" t="n">
         <v>0</v>
       </c>
+      <c r="W158" t="n">
+        <v>25.2</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -11271,6 +11747,9 @@
       <c r="V159" t="n">
         <v>0</v>
       </c>
+      <c r="W159" t="n">
+        <v>27.1</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -11339,6 +11818,9 @@
       <c r="V160" t="n">
         <v>0</v>
       </c>
+      <c r="W160" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -11407,6 +11889,9 @@
       <c r="V161" t="n">
         <v>0</v>
       </c>
+      <c r="W161" t="n">
+        <v>41.9</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -11475,6 +11960,9 @@
       <c r="V162" t="n">
         <v>0</v>
       </c>
+      <c r="W162" t="n">
+        <v>35.6</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -11543,6 +12031,9 @@
       <c r="V163" t="n">
         <v>0</v>
       </c>
+      <c r="W163" t="n">
+        <v>53.4</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -11611,6 +12102,9 @@
       <c r="V164" t="n">
         <v>0</v>
       </c>
+      <c r="W164" t="n">
+        <v>34</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -11679,6 +12173,9 @@
       <c r="V165" t="n">
         <v>0</v>
       </c>
+      <c r="W165" t="n">
+        <v>7.1</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -11747,6 +12244,9 @@
       <c r="V166" t="n">
         <v>1</v>
       </c>
+      <c r="W166" t="n">
+        <v>38.5</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -11815,6 +12315,9 @@
       <c r="V167" t="n">
         <v>0</v>
       </c>
+      <c r="W167" t="n">
+        <v>6.8</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -11883,6 +12386,9 @@
       <c r="V168" t="n">
         <v>1</v>
       </c>
+      <c r="W168" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -11951,6 +12457,9 @@
       <c r="V169" t="n">
         <v>0</v>
       </c>
+      <c r="W169" t="n">
+        <v>58.1</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -12019,6 +12528,9 @@
       <c r="V170" t="n">
         <v>0</v>
       </c>
+      <c r="W170" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -12087,6 +12599,9 @@
       <c r="V171" t="n">
         <v>1</v>
       </c>
+      <c r="W171" t="n">
+        <v>39.3</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -12155,6 +12670,9 @@
       <c r="V172" t="n">
         <v>0</v>
       </c>
+      <c r="W172" t="n">
+        <v>19.5</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -12223,6 +12741,9 @@
       <c r="V173" t="n">
         <v>0</v>
       </c>
+      <c r="W173" t="n">
+        <v>29.7</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -12291,6 +12812,9 @@
       <c r="V174" t="n">
         <v>0</v>
       </c>
+      <c r="W174" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -12359,6 +12883,9 @@
       <c r="V175" t="n">
         <v>0</v>
       </c>
+      <c r="W175" t="n">
+        <v>35.7</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -12427,6 +12954,9 @@
       <c r="V176" t="n">
         <v>0</v>
       </c>
+      <c r="W176" t="n">
+        <v>3.4</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -12495,6 +13025,9 @@
       <c r="V177" t="n">
         <v>0</v>
       </c>
+      <c r="W177" t="n">
+        <v>23.4</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -12563,6 +13096,9 @@
       <c r="V178" t="n">
         <v>0</v>
       </c>
+      <c r="W178" t="n">
+        <v>27.1</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -12631,6 +13167,9 @@
       <c r="V179" t="n">
         <v>1</v>
       </c>
+      <c r="W179" t="n">
+        <v>39.4</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -12699,6 +13238,9 @@
       <c r="V180" t="n">
         <v>0</v>
       </c>
+      <c r="W180" t="n">
+        <v>27.8</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -12767,6 +13309,9 @@
       <c r="V181" t="n">
         <v>1</v>
       </c>
+      <c r="W181" t="n">
+        <v>38.7</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -12835,6 +13380,9 @@
       <c r="V182" t="n">
         <v>0</v>
       </c>
+      <c r="W182" t="n">
+        <v>15.3</v>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -12903,6 +13451,9 @@
       <c r="V183" t="n">
         <v>0</v>
       </c>
+      <c r="W183" t="n">
+        <v>46.8</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -12971,6 +13522,9 @@
       <c r="V184" t="n">
         <v>0</v>
       </c>
+      <c r="W184" t="n">
+        <v>14.5</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -13039,6 +13593,9 @@
       <c r="V185" t="n">
         <v>1</v>
       </c>
+      <c r="W185" t="n">
+        <v>39.5</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -13107,6 +13664,9 @@
       <c r="V186" t="n">
         <v>0</v>
       </c>
+      <c r="W186" t="n">
+        <v>14.5</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -13175,6 +13735,9 @@
       <c r="V187" t="n">
         <v>0</v>
       </c>
+      <c r="W187" t="n">
+        <v>17.3</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -13243,6 +13806,9 @@
       <c r="V188" t="n">
         <v>0</v>
       </c>
+      <c r="W188" t="n">
+        <v>15.5</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -13311,6 +13877,9 @@
       <c r="V189" t="n">
         <v>0</v>
       </c>
+      <c r="W189" t="n">
+        <v>25.2</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -13379,6 +13948,9 @@
       <c r="V190" t="n">
         <v>0</v>
       </c>
+      <c r="W190" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -13447,6 +14019,9 @@
       <c r="V191" t="n">
         <v>0</v>
       </c>
+      <c r="W191" t="n">
+        <v>18.9</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -13515,6 +14090,9 @@
       <c r="V192" t="n">
         <v>0</v>
       </c>
+      <c r="W192" t="n">
+        <v>1.7</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -13583,6 +14161,9 @@
       <c r="V193" t="n">
         <v>0</v>
       </c>
+      <c r="W193" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -13651,6 +14232,9 @@
       <c r="V194" t="n">
         <v>0</v>
       </c>
+      <c r="W194" t="n">
+        <v>24.9</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -13719,6 +14303,9 @@
       <c r="V195" t="n">
         <v>0</v>
       </c>
+      <c r="W195" t="n">
+        <v>38.4</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -13787,6 +14374,9 @@
       <c r="V196" t="n">
         <v>0</v>
       </c>
+      <c r="W196" t="n">
+        <v>30.1</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -13855,6 +14445,9 @@
       <c r="V197" t="n">
         <v>0</v>
       </c>
+      <c r="W197" t="n">
+        <v>17.2</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -13923,6 +14516,9 @@
       <c r="V198" t="n">
         <v>0</v>
       </c>
+      <c r="W198" t="n">
+        <v>11.2</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -13991,6 +14587,9 @@
       <c r="V199" t="n">
         <v>0</v>
       </c>
+      <c r="W199" t="n">
+        <v>9.1</v>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -14059,6 +14658,9 @@
       <c r="V200" t="n">
         <v>0</v>
       </c>
+      <c r="W200" t="n">
+        <v>37.3</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -14127,6 +14729,9 @@
       <c r="V201" t="n">
         <v>1</v>
       </c>
+      <c r="W201" t="n">
+        <v>46.5</v>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -14195,6 +14800,9 @@
       <c r="V202" t="n">
         <v>1</v>
       </c>
+      <c r="W202" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="n">
@@ -14263,6 +14871,9 @@
       <c r="V203" t="n">
         <v>0</v>
       </c>
+      <c r="W203" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -14331,6 +14942,9 @@
       <c r="V204" t="n">
         <v>1</v>
       </c>
+      <c r="W204" t="n">
+        <v>16.5</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="n">
@@ -14399,6 +15013,9 @@
       <c r="V205" t="n">
         <v>0</v>
       </c>
+      <c r="W205" t="n">
+        <v>37.1</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -14467,6 +15084,9 @@
       <c r="V206" t="n">
         <v>0</v>
       </c>
+      <c r="W206" t="n">
+        <v>39.3</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -14535,6 +15155,9 @@
       <c r="V207" t="n">
         <v>0</v>
       </c>
+      <c r="W207" t="n">
+        <v>13.3</v>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -14603,6 +15226,9 @@
       <c r="V208" t="n">
         <v>1</v>
       </c>
+      <c r="W208" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="n">
@@ -14671,6 +15297,9 @@
       <c r="V209" t="n">
         <v>0</v>
       </c>
+      <c r="W209" t="n">
+        <v>12.1</v>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="n">
@@ -14739,6 +15368,9 @@
       <c r="V210" t="n">
         <v>0</v>
       </c>
+      <c r="W210" t="n">
+        <v>17.4</v>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -14807,6 +15439,9 @@
       <c r="V211" t="n">
         <v>1</v>
       </c>
+      <c r="W211" t="n">
+        <v>29.3</v>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="n">
@@ -14875,6 +15510,9 @@
       <c r="V212" t="n">
         <v>1</v>
       </c>
+      <c r="W212" t="n">
+        <v>25.3</v>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -14943,6 +15581,9 @@
       <c r="V213" t="n">
         <v>0</v>
       </c>
+      <c r="W213" t="n">
+        <v>16.6</v>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="n">
@@ -15011,6 +15652,9 @@
       <c r="V214" t="n">
         <v>0</v>
       </c>
+      <c r="W214" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="n">
@@ -15079,6 +15723,9 @@
       <c r="V215" t="n">
         <v>0</v>
       </c>
+      <c r="W215" t="n">
+        <v>31</v>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="n">
@@ -15147,6 +15794,9 @@
       <c r="V216" t="n">
         <v>0</v>
       </c>
+      <c r="W216" t="n">
+        <v>33</v>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="n">
@@ -15215,6 +15865,9 @@
       <c r="V217" t="n">
         <v>0</v>
       </c>
+      <c r="W217" t="n">
+        <v>38.6</v>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="n">
@@ -15283,6 +15936,9 @@
       <c r="V218" t="n">
         <v>1</v>
       </c>
+      <c r="W218" t="n">
+        <v>12.5</v>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="n">
@@ -15351,6 +16007,9 @@
       <c r="V219" t="n">
         <v>0</v>
       </c>
+      <c r="W219" t="n">
+        <v>34.1</v>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="n">
@@ -15419,6 +16078,9 @@
       <c r="V220" t="n">
         <v>0</v>
       </c>
+      <c r="W220" t="n">
+        <v>11.8</v>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="n">
@@ -15487,6 +16149,9 @@
       <c r="V221" t="n">
         <v>0</v>
       </c>
+      <c r="W221" t="n">
+        <v>34.5</v>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="n">
@@ -15555,6 +16220,9 @@
       <c r="V222" t="n">
         <v>0</v>
       </c>
+      <c r="W222" t="n">
+        <v>36.7</v>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -15623,6 +16291,9 @@
       <c r="V223" t="n">
         <v>0</v>
       </c>
+      <c r="W223" t="n">
+        <v>15.3</v>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="n">
@@ -15691,6 +16362,9 @@
       <c r="V224" t="n">
         <v>0</v>
       </c>
+      <c r="W224" t="n">
+        <v>18.9</v>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="n">
@@ -15759,6 +16433,9 @@
       <c r="V225" t="n">
         <v>0</v>
       </c>
+      <c r="W225" t="n">
+        <v>35.5</v>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="n">
@@ -15827,6 +16504,9 @@
       <c r="V226" t="n">
         <v>0</v>
       </c>
+      <c r="W226" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="n">
@@ -15895,6 +16575,9 @@
       <c r="V227" t="n">
         <v>0</v>
       </c>
+      <c r="W227" t="n">
+        <v>26.3</v>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="n">
@@ -15963,6 +16646,9 @@
       <c r="V228" t="n">
         <v>0</v>
       </c>
+      <c r="W228" t="n">
+        <v>30.6</v>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -16031,6 +16717,9 @@
       <c r="V229" t="n">
         <v>0</v>
       </c>
+      <c r="W229" t="n">
+        <v>31.7</v>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="n">
@@ -16099,6 +16788,9 @@
       <c r="V230" t="n">
         <v>1</v>
       </c>
+      <c r="W230" t="n">
+        <v>17.9</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="n">
@@ -16167,6 +16859,9 @@
       <c r="V231" t="n">
         <v>0</v>
       </c>
+      <c r="W231" t="n">
+        <v>7.8</v>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="n">
@@ -16235,6 +16930,9 @@
       <c r="V232" t="n">
         <v>0</v>
       </c>
+      <c r="W232" t="n">
+        <v>16.6</v>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="n">
@@ -16303,6 +17001,9 @@
       <c r="V233" t="n">
         <v>1</v>
       </c>
+      <c r="W233" t="n">
+        <v>39</v>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="n">
@@ -16371,6 +17072,9 @@
       <c r="V234" t="n">
         <v>0</v>
       </c>
+      <c r="W234" t="n">
+        <v>6.1</v>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="n">
@@ -16439,6 +17143,9 @@
       <c r="V235" t="n">
         <v>1</v>
       </c>
+      <c r="W235" t="n">
+        <v>13.1</v>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="n">
@@ -16507,6 +17214,9 @@
       <c r="V236" t="n">
         <v>0</v>
       </c>
+      <c r="W236" t="n">
+        <v>19.4</v>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="n">
@@ -16575,6 +17285,9 @@
       <c r="V237" t="n">
         <v>0</v>
       </c>
+      <c r="W237" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="n">
@@ -16643,6 +17356,9 @@
       <c r="V238" t="n">
         <v>0</v>
       </c>
+      <c r="W238" t="n">
+        <v>27.2</v>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="n">
@@ -16711,6 +17427,9 @@
       <c r="V239" t="n">
         <v>1</v>
       </c>
+      <c r="W239" t="n">
+        <v>11.5</v>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="n">
@@ -16779,6 +17498,9 @@
       <c r="V240" t="n">
         <v>1</v>
       </c>
+      <c r="W240" t="n">
+        <v>23.3</v>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="n">
@@ -16847,6 +17569,9 @@
       <c r="V241" t="n">
         <v>1</v>
       </c>
+      <c r="W241" t="n">
+        <v>27.6</v>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="n">
@@ -16915,6 +17640,9 @@
       <c r="V242" t="n">
         <v>1</v>
       </c>
+      <c r="W242" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="n">
@@ -16983,6 +17711,9 @@
       <c r="V243" t="n">
         <v>1</v>
       </c>
+      <c r="W243" t="n">
+        <v>29.4</v>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="n">
@@ -17051,6 +17782,9 @@
       <c r="V244" t="n">
         <v>1</v>
       </c>
+      <c r="W244" t="n">
+        <v>18.5</v>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="n">
@@ -17119,6 +17853,9 @@
       <c r="V245" t="n">
         <v>0</v>
       </c>
+      <c r="W245" t="n">
+        <v>33.3</v>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="n">
@@ -17187,6 +17924,9 @@
       <c r="V246" t="n">
         <v>0</v>
       </c>
+      <c r="W246" t="n">
+        <v>43.3</v>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="n">
@@ -17255,6 +17995,9 @@
       <c r="V247" t="n">
         <v>1</v>
       </c>
+      <c r="W247" t="n">
+        <v>15.8</v>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="n">
@@ -17323,6 +18066,9 @@
       <c r="V248" t="n">
         <v>0</v>
       </c>
+      <c r="W248" t="n">
+        <v>33.6</v>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="n">
@@ -17391,6 +18137,9 @@
       <c r="V249" t="n">
         <v>0</v>
       </c>
+      <c r="W249" t="n">
+        <v>36.2</v>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="n">
@@ -17459,6 +18208,9 @@
       <c r="V250" t="n">
         <v>0</v>
       </c>
+      <c r="W250" t="n">
+        <v>48.1</v>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="n">
@@ -17527,6 +18279,9 @@
       <c r="V251" t="n">
         <v>0</v>
       </c>
+      <c r="W251" t="n">
+        <v>17.1</v>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="n">
@@ -17595,6 +18350,9 @@
       <c r="V252" t="n">
         <v>1</v>
       </c>
+      <c r="W252" t="n">
+        <v>40.7</v>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="n">
@@ -17663,6 +18421,9 @@
       <c r="V253" t="n">
         <v>0</v>
       </c>
+      <c r="W253" t="n">
+        <v>18.5</v>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="n">
@@ -17731,6 +18492,9 @@
       <c r="V254" t="n">
         <v>0</v>
       </c>
+      <c r="W254" t="n">
+        <v>24.3</v>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="n">
@@ -17799,6 +18563,9 @@
       <c r="V255" t="n">
         <v>0</v>
       </c>
+      <c r="W255" t="n">
+        <v>16.2</v>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="n">
@@ -17867,6 +18634,9 @@
       <c r="V256" t="n">
         <v>0</v>
       </c>
+      <c r="W256" t="n">
+        <v>25.8</v>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="n">
@@ -17935,6 +18705,9 @@
       <c r="V257" t="n">
         <v>0</v>
       </c>
+      <c r="W257" t="n">
+        <v>32.6</v>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="n">
@@ -18003,6 +18776,9 @@
       <c r="V258" t="n">
         <v>1</v>
       </c>
+      <c r="W258" t="n">
+        <v>27.4</v>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="n">
@@ -18071,6 +18847,9 @@
       <c r="V259" t="n">
         <v>0</v>
       </c>
+      <c r="W259" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="n">
@@ -18139,6 +18918,9 @@
       <c r="V260" t="n">
         <v>0</v>
       </c>
+      <c r="W260" t="n">
+        <v>34.9</v>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="n">
@@ -18207,6 +18989,9 @@
       <c r="V261" t="n">
         <v>0</v>
       </c>
+      <c r="W261" t="n">
+        <v>43.3</v>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="n">
@@ -18275,6 +19060,9 @@
       <c r="V262" t="n">
         <v>1</v>
       </c>
+      <c r="W262" t="n">
+        <v>16.5</v>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="n">
@@ -18343,6 +19131,9 @@
       <c r="V263" t="n">
         <v>0</v>
       </c>
+      <c r="W263" t="n">
+        <v>4.5</v>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="n">
@@ -18411,6 +19202,9 @@
       <c r="V264" t="n">
         <v>1</v>
       </c>
+      <c r="W264" t="n">
+        <v>7.5</v>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="n">
@@ -18479,6 +19273,9 @@
       <c r="V265" t="n">
         <v>0</v>
       </c>
+      <c r="W265" t="n">
+        <v>32.6</v>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="n">
@@ -18547,6 +19344,9 @@
       <c r="V266" t="n">
         <v>0</v>
       </c>
+      <c r="W266" t="n">
+        <v>30.6</v>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="n">
@@ -18615,6 +19415,9 @@
       <c r="V267" t="n">
         <v>0</v>
       </c>
+      <c r="W267" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="n">
@@ -18683,6 +19486,9 @@
       <c r="V268" t="n">
         <v>0</v>
       </c>
+      <c r="W268" t="n">
+        <v>30.6</v>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="n">
@@ -18751,6 +19557,9 @@
       <c r="V269" t="n">
         <v>0</v>
       </c>
+      <c r="W269" t="n">
+        <v>12.5</v>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="n">
@@ -18819,6 +19628,9 @@
       <c r="V270" t="n">
         <v>0</v>
       </c>
+      <c r="W270" t="n">
+        <v>1.8</v>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="n">
@@ -18887,6 +19699,9 @@
       <c r="V271" t="n">
         <v>0</v>
       </c>
+      <c r="W271" t="n">
+        <v>31.7</v>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="n">
@@ -18955,6 +19770,9 @@
       <c r="V272" t="n">
         <v>0</v>
       </c>
+      <c r="W272" t="n">
+        <v>34.3</v>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="n">
@@ -19023,6 +19841,9 @@
       <c r="V273" t="n">
         <v>1</v>
       </c>
+      <c r="W273" t="n">
+        <v>16.3</v>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="n">
@@ -19091,6 +19912,9 @@
       <c r="V274" t="n">
         <v>0</v>
       </c>
+      <c r="W274" t="n">
+        <v>35</v>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="n">
@@ -19159,6 +19983,9 @@
       <c r="V275" t="n">
         <v>1</v>
       </c>
+      <c r="W275" t="n">
+        <v>17.4</v>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="n">
@@ -19227,6 +20054,9 @@
       <c r="V276" t="n">
         <v>0</v>
       </c>
+      <c r="W276" t="n">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="n">
@@ -19295,6 +20125,9 @@
       <c r="V277" t="n">
         <v>1</v>
       </c>
+      <c r="W277" t="n">
+        <v>29.2</v>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="n">
@@ -19363,6 +20196,9 @@
       <c r="V278" t="n">
         <v>0</v>
       </c>
+      <c r="W278" t="n">
+        <v>13.1</v>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="n">
@@ -19431,6 +20267,9 @@
       <c r="V279" t="n">
         <v>0</v>
       </c>
+      <c r="W279" t="n">
+        <v>28.4</v>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="n">
@@ -19499,6 +20338,9 @@
       <c r="V280" t="n">
         <v>0</v>
       </c>
+      <c r="W280" t="n">
+        <v>39.3</v>
+      </c>
     </row>
     <row r="281">
       <c r="A281" t="n">
@@ -19567,6 +20409,9 @@
       <c r="V281" t="n">
         <v>0</v>
       </c>
+      <c r="W281" t="n">
+        <v>38.1</v>
+      </c>
     </row>
     <row r="282">
       <c r="A282" t="n">
@@ -19635,6 +20480,9 @@
       <c r="V282" t="n">
         <v>0</v>
       </c>
+      <c r="W282" t="n">
+        <v>23.9</v>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="n">
@@ -19703,6 +20551,9 @@
       <c r="V283" t="n">
         <v>1</v>
       </c>
+      <c r="W283" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="284">
       <c r="A284" t="n">
@@ -19771,6 +20622,9 @@
       <c r="V284" t="n">
         <v>1</v>
       </c>
+      <c r="W284" t="n">
+        <v>30.9</v>
+      </c>
     </row>
     <row r="285">
       <c r="A285" t="n">
@@ -19839,6 +20693,9 @@
       <c r="V285" t="n">
         <v>0</v>
       </c>
+      <c r="W285" t="n">
+        <v>32.1</v>
+      </c>
     </row>
     <row r="286">
       <c r="A286" t="n">
@@ -19907,6 +20764,9 @@
       <c r="V286" t="n">
         <v>0</v>
       </c>
+      <c r="W286" t="n">
+        <v>8.1</v>
+      </c>
     </row>
     <row r="287">
       <c r="A287" t="n">
@@ -19975,6 +20835,9 @@
       <c r="V287" t="n">
         <v>0</v>
       </c>
+      <c r="W287" t="n">
+        <v>31.8</v>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="n">
@@ -20043,6 +20906,9 @@
       <c r="V288" t="n">
         <v>0</v>
       </c>
+      <c r="W288" t="n">
+        <v>9.800000000000001</v>
+      </c>
     </row>
     <row r="289">
       <c r="A289" t="n">
@@ -20111,6 +20977,9 @@
       <c r="V289" t="n">
         <v>0</v>
       </c>
+      <c r="W289" t="n">
+        <v>14.5</v>
+      </c>
     </row>
     <row r="290">
       <c r="A290" t="n">
@@ -20179,6 +21048,9 @@
       <c r="V290" t="n">
         <v>0</v>
       </c>
+      <c r="W290" t="n">
+        <v>24.9</v>
+      </c>
     </row>
     <row r="291">
       <c r="A291" t="n">
@@ -20247,6 +21119,9 @@
       <c r="V291" t="n">
         <v>0</v>
       </c>
+      <c r="W291" t="n">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="292">
       <c r="A292" t="n">
@@ -20315,6 +21190,9 @@
       <c r="V292" t="n">
         <v>0</v>
       </c>
+      <c r="W292" t="n">
+        <v>40.8</v>
+      </c>
     </row>
     <row r="293">
       <c r="A293" t="n">
@@ -20383,6 +21261,9 @@
       <c r="V293" t="n">
         <v>0</v>
       </c>
+      <c r="W293" t="n">
+        <v>35.6</v>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="n">
@@ -20451,6 +21332,9 @@
       <c r="V294" t="n">
         <v>0</v>
       </c>
+      <c r="W294" t="n">
+        <v>20.6</v>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="n">
@@ -20519,6 +21403,9 @@
       <c r="V295" t="n">
         <v>0</v>
       </c>
+      <c r="W295" t="n">
+        <v>15.1</v>
+      </c>
     </row>
     <row r="296">
       <c r="A296" t="n">
@@ -20587,6 +21474,9 @@
       <c r="V296" t="n">
         <v>1</v>
       </c>
+      <c r="W296" t="n">
+        <v>19.5</v>
+      </c>
     </row>
     <row r="297">
       <c r="A297" t="n">
@@ -20655,6 +21545,9 @@
       <c r="V297" t="n">
         <v>0</v>
       </c>
+      <c r="W297" t="n">
+        <v>29.4</v>
+      </c>
     </row>
     <row r="298">
       <c r="A298" t="n">
@@ -20723,6 +21616,9 @@
       <c r="V298" t="n">
         <v>1</v>
       </c>
+      <c r="W298" t="n">
+        <v>32.1</v>
+      </c>
     </row>
     <row r="299">
       <c r="A299" t="n">
@@ -20791,6 +21687,9 @@
       <c r="V299" t="n">
         <v>0</v>
       </c>
+      <c r="W299" t="n">
+        <v>27.2</v>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="n">
@@ -20859,6 +21758,9 @@
       <c r="V300" t="n">
         <v>0</v>
       </c>
+      <c r="W300" t="n">
+        <v>32.5</v>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="n">
@@ -20927,6 +21829,9 @@
       <c r="V301" t="n">
         <v>0</v>
       </c>
+      <c r="W301" t="n">
+        <v>36.5</v>
+      </c>
     </row>
     <row r="302">
       <c r="A302" t="n">
@@ -20995,6 +21900,9 @@
       <c r="V302" t="n">
         <v>1</v>
       </c>
+      <c r="W302" t="n">
+        <v>34.2</v>
+      </c>
     </row>
     <row r="303">
       <c r="A303" t="n">
@@ -21063,6 +21971,9 @@
       <c r="V303" t="n">
         <v>0</v>
       </c>
+      <c r="W303" t="n">
+        <v>36.6</v>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="n">
@@ -21131,6 +22042,9 @@
       <c r="V304" t="n">
         <v>0</v>
       </c>
+      <c r="W304" t="n">
+        <v>14.8</v>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="n">
@@ -21199,6 +22113,9 @@
       <c r="V305" t="n">
         <v>0</v>
       </c>
+      <c r="W305" t="n">
+        <v>38.2</v>
+      </c>
     </row>
     <row r="306">
       <c r="A306" t="n">
@@ -21267,6 +22184,9 @@
       <c r="V306" t="n">
         <v>1</v>
       </c>
+      <c r="W306" t="n">
+        <v>12.7</v>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="n">
@@ -21335,6 +22255,9 @@
       <c r="V307" t="n">
         <v>0</v>
       </c>
+      <c r="W307" t="n">
+        <v>22.4</v>
+      </c>
     </row>
     <row r="308">
       <c r="A308" t="n">
@@ -21403,6 +22326,9 @@
       <c r="V308" t="n">
         <v>1</v>
       </c>
+      <c r="W308" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="309">
       <c r="A309" t="n">
@@ -21471,6 +22397,9 @@
       <c r="V309" t="n">
         <v>0</v>
       </c>
+      <c r="W309" t="n">
+        <v>26.9</v>
+      </c>
     </row>
     <row r="310">
       <c r="A310" t="n">
@@ -21539,6 +22468,9 @@
       <c r="V310" t="n">
         <v>0</v>
       </c>
+      <c r="W310" t="n">
+        <v>37.8</v>
+      </c>
     </row>
     <row r="311">
       <c r="A311" t="n">
@@ -21607,6 +22539,9 @@
       <c r="V311" t="n">
         <v>0</v>
       </c>
+      <c r="W311" t="n">
+        <v>18.8</v>
+      </c>
     </row>
     <row r="312">
       <c r="A312" t="n">
@@ -21675,6 +22610,9 @@
       <c r="V312" t="n">
         <v>0</v>
       </c>
+      <c r="W312" t="n">
+        <v>16.9</v>
+      </c>
     </row>
     <row r="313">
       <c r="A313" t="n">
@@ -21743,6 +22681,9 @@
       <c r="V313" t="n">
         <v>1</v>
       </c>
+      <c r="W313" t="n">
+        <v>25.2</v>
+      </c>
     </row>
     <row r="314">
       <c r="A314" t="n">
@@ -21811,6 +22752,9 @@
       <c r="V314" t="n">
         <v>1</v>
       </c>
+      <c r="W314" t="n">
+        <v>7.7</v>
+      </c>
     </row>
     <row r="315">
       <c r="A315" t="n">
@@ -21879,6 +22823,9 @@
       <c r="V315" t="n">
         <v>0</v>
       </c>
+      <c r="W315" t="n">
+        <v>6.6</v>
+      </c>
     </row>
     <row r="316">
       <c r="A316" t="n">
@@ -21947,6 +22894,9 @@
       <c r="V316" t="n">
         <v>0</v>
       </c>
+      <c r="W316" t="n">
+        <v>14.2</v>
+      </c>
     </row>
     <row r="317">
       <c r="A317" t="n">
@@ -22015,6 +22965,9 @@
       <c r="V317" t="n">
         <v>0</v>
       </c>
+      <c r="W317" t="n">
+        <v>27.2</v>
+      </c>
     </row>
     <row r="318">
       <c r="A318" t="n">
@@ -22083,6 +23036,9 @@
       <c r="V318" t="n">
         <v>0</v>
       </c>
+      <c r="W318" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="319">
       <c r="A319" t="n">
@@ -22151,6 +23107,9 @@
       <c r="V319" t="n">
         <v>1</v>
       </c>
+      <c r="W319" t="n">
+        <v>17.6</v>
+      </c>
     </row>
     <row r="320">
       <c r="A320" t="n">
@@ -22219,6 +23178,9 @@
       <c r="V320" t="n">
         <v>0</v>
       </c>
+      <c r="W320" t="n">
+        <v>23.2</v>
+      </c>
     </row>
     <row r="321">
       <c r="A321" t="n">
@@ -22287,6 +23249,9 @@
       <c r="V321" t="n">
         <v>0</v>
       </c>
+      <c r="W321" t="n">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="322">
       <c r="A322" t="n">
@@ -22355,6 +23320,9 @@
       <c r="V322" t="n">
         <v>0</v>
       </c>
+      <c r="W322" t="n">
+        <v>11.8</v>
+      </c>
     </row>
     <row r="323">
       <c r="A323" t="n">
@@ -22423,6 +23391,9 @@
       <c r="V323" t="n">
         <v>1</v>
       </c>
+      <c r="W323" t="n">
+        <v>18.2</v>
+      </c>
     </row>
     <row r="324">
       <c r="A324" t="n">
@@ -22491,6 +23462,9 @@
       <c r="V324" t="n">
         <v>0</v>
       </c>
+      <c r="W324" t="n">
+        <v>11.8</v>
+      </c>
     </row>
     <row r="325">
       <c r="A325" t="n">
@@ -22559,6 +23533,9 @@
       <c r="V325" t="n">
         <v>1</v>
       </c>
+      <c r="W325" t="n">
+        <v>40.4</v>
+      </c>
     </row>
     <row r="326">
       <c r="A326" t="n">
@@ -22627,6 +23604,9 @@
       <c r="V326" t="n">
         <v>0</v>
       </c>
+      <c r="W326" t="n">
+        <v>19.2</v>
+      </c>
     </row>
     <row r="327">
       <c r="A327" t="n">
@@ -22695,6 +23675,9 @@
       <c r="V327" t="n">
         <v>0</v>
       </c>
+      <c r="W327" t="n">
+        <v>7.7</v>
+      </c>
     </row>
     <row r="328">
       <c r="A328" t="n">
@@ -22763,6 +23746,9 @@
       <c r="V328" t="n">
         <v>0</v>
       </c>
+      <c r="W328" t="n">
+        <v>7.9</v>
+      </c>
     </row>
     <row r="329">
       <c r="A329" t="n">
@@ -22831,6 +23817,9 @@
       <c r="V329" t="n">
         <v>0</v>
       </c>
+      <c r="W329" t="n">
+        <v>6.3</v>
+      </c>
     </row>
     <row r="330">
       <c r="A330" t="n">
@@ -22899,6 +23888,9 @@
       <c r="V330" t="n">
         <v>0</v>
       </c>
+      <c r="W330" t="n">
+        <v>22.9</v>
+      </c>
     </row>
     <row r="331">
       <c r="A331" t="n">
@@ -22967,6 +23959,9 @@
       <c r="V331" t="n">
         <v>1</v>
       </c>
+      <c r="W331" t="n">
+        <v>23.2</v>
+      </c>
     </row>
     <row r="332">
       <c r="A332" t="n">
@@ -23035,6 +24030,9 @@
       <c r="V332" t="n">
         <v>0</v>
       </c>
+      <c r="W332" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="333">
       <c r="A333" t="n">
@@ -23103,6 +24101,9 @@
       <c r="V333" t="n">
         <v>0</v>
       </c>
+      <c r="W333" t="n">
+        <v>32.1</v>
+      </c>
     </row>
     <row r="334">
       <c r="A334" t="n">
@@ -23171,6 +24172,9 @@
       <c r="V334" t="n">
         <v>0</v>
       </c>
+      <c r="W334" t="n">
+        <v>31.8</v>
+      </c>
     </row>
     <row r="335">
       <c r="A335" t="n">
@@ -23239,6 +24243,9 @@
       <c r="V335" t="n">
         <v>0</v>
       </c>
+      <c r="W335" t="n">
+        <v>13.9</v>
+      </c>
     </row>
     <row r="336">
       <c r="A336" t="n">
@@ -23307,6 +24314,9 @@
       <c r="V336" t="n">
         <v>1</v>
       </c>
+      <c r="W336" t="n">
+        <v>35.7</v>
+      </c>
     </row>
     <row r="337">
       <c r="A337" t="n">
@@ -23375,6 +24385,9 @@
       <c r="V337" t="n">
         <v>0</v>
       </c>
+      <c r="W337" t="n">
+        <v>33.5</v>
+      </c>
     </row>
     <row r="338">
       <c r="A338" t="n">
@@ -23443,6 +24456,9 @@
       <c r="V338" t="n">
         <v>0</v>
       </c>
+      <c r="W338" t="n">
+        <v>26.2</v>
+      </c>
     </row>
     <row r="339">
       <c r="A339" t="n">
@@ -23511,6 +24527,9 @@
       <c r="V339" t="n">
         <v>1</v>
       </c>
+      <c r="W339" t="n">
+        <v>34.5</v>
+      </c>
     </row>
     <row r="340">
       <c r="A340" t="n">
@@ -23579,6 +24598,9 @@
       <c r="V340" t="n">
         <v>0</v>
       </c>
+      <c r="W340" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="341">
       <c r="A341" t="n">
@@ -23647,6 +24669,9 @@
       <c r="V341" t="n">
         <v>0</v>
       </c>
+      <c r="W341" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="342">
       <c r="A342" t="n">
@@ -23715,6 +24740,9 @@
       <c r="V342" t="n">
         <v>0</v>
       </c>
+      <c r="W342" t="n">
+        <v>33</v>
+      </c>
     </row>
     <row r="343">
       <c r="A343" t="n">
@@ -23783,6 +24811,9 @@
       <c r="V343" t="n">
         <v>0</v>
       </c>
+      <c r="W343" t="n">
+        <v>15.4</v>
+      </c>
     </row>
     <row r="344">
       <c r="A344" t="n">
@@ -23851,6 +24882,9 @@
       <c r="V344" t="n">
         <v>0</v>
       </c>
+      <c r="W344" t="n">
+        <v>20.6</v>
+      </c>
     </row>
     <row r="345">
       <c r="A345" t="n">
@@ -23919,6 +24953,9 @@
       <c r="V345" t="n">
         <v>1</v>
       </c>
+      <c r="W345" t="n">
+        <v>11.6</v>
+      </c>
     </row>
     <row r="346">
       <c r="A346" t="n">
@@ -23987,6 +25024,9 @@
       <c r="V346" t="n">
         <v>1</v>
       </c>
+      <c r="W346" t="n">
+        <v>17.5</v>
+      </c>
     </row>
     <row r="347">
       <c r="A347" t="n">
@@ -24055,6 +25095,9 @@
       <c r="V347" t="n">
         <v>0</v>
       </c>
+      <c r="W347" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="348">
       <c r="A348" t="n">
@@ -24123,6 +25166,9 @@
       <c r="V348" t="n">
         <v>0</v>
       </c>
+      <c r="W348" t="n">
+        <v>15.6</v>
+      </c>
     </row>
     <row r="349">
       <c r="A349" t="n">
@@ -24191,6 +25237,9 @@
       <c r="V349" t="n">
         <v>0</v>
       </c>
+      <c r="W349" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="350">
       <c r="A350" t="n">
@@ -24259,6 +25308,9 @@
       <c r="V350" t="n">
         <v>0</v>
       </c>
+      <c r="W350" t="n">
+        <v>38.1</v>
+      </c>
     </row>
     <row r="351">
       <c r="A351" t="n">
@@ -24327,6 +25379,9 @@
       <c r="V351" t="n">
         <v>0</v>
       </c>
+      <c r="W351" t="n">
+        <v>27.9</v>
+      </c>
     </row>
     <row r="352">
       <c r="A352" t="n">
@@ -24395,6 +25450,9 @@
       <c r="V352" t="n">
         <v>1</v>
       </c>
+      <c r="W352" t="n">
+        <v>39</v>
+      </c>
     </row>
     <row r="353">
       <c r="A353" t="n">
@@ -24463,6 +25521,9 @@
       <c r="V353" t="n">
         <v>0</v>
       </c>
+      <c r="W353" t="n">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="354">
       <c r="A354" t="n">
@@ -24531,6 +25592,9 @@
       <c r="V354" t="n">
         <v>1</v>
       </c>
+      <c r="W354" t="n">
+        <v>14.1</v>
+      </c>
     </row>
     <row r="355">
       <c r="A355" t="n">
@@ -24599,6 +25663,9 @@
       <c r="V355" t="n">
         <v>0</v>
       </c>
+      <c r="W355" t="n">
+        <v>24.1</v>
+      </c>
     </row>
     <row r="356">
       <c r="A356" t="n">
@@ -24667,6 +25734,9 @@
       <c r="V356" t="n">
         <v>0</v>
       </c>
+      <c r="W356" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="357">
       <c r="A357" t="n">
@@ -24735,6 +25805,9 @@
       <c r="V357" t="n">
         <v>0</v>
       </c>
+      <c r="W357" t="n">
+        <v>25.7</v>
+      </c>
     </row>
     <row r="358">
       <c r="A358" t="n">
@@ -24803,6 +25876,9 @@
       <c r="V358" t="n">
         <v>0</v>
       </c>
+      <c r="W358" t="n">
+        <v>10.8</v>
+      </c>
     </row>
     <row r="359">
       <c r="A359" t="n">
@@ -24871,6 +25947,9 @@
       <c r="V359" t="n">
         <v>1</v>
       </c>
+      <c r="W359" t="n">
+        <v>2.8</v>
+      </c>
     </row>
     <row r="360">
       <c r="A360" t="n">
@@ -24939,6 +26018,9 @@
       <c r="V360" t="n">
         <v>0</v>
       </c>
+      <c r="W360" t="n">
+        <v>11.8</v>
+      </c>
     </row>
     <row r="361">
       <c r="A361" t="n">
@@ -25007,6 +26089,9 @@
       <c r="V361" t="n">
         <v>0</v>
       </c>
+      <c r="W361" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="362">
       <c r="A362" t="n">
@@ -25075,6 +26160,9 @@
       <c r="V362" t="n">
         <v>0</v>
       </c>
+      <c r="W362" t="n">
+        <v>39.5</v>
+      </c>
     </row>
     <row r="363">
       <c r="A363" t="n">
@@ -25143,6 +26231,9 @@
       <c r="V363" t="n">
         <v>1</v>
       </c>
+      <c r="W363" t="n">
+        <v>42.7</v>
+      </c>
     </row>
     <row r="364">
       <c r="A364" t="n">
@@ -25211,6 +26302,9 @@
       <c r="V364" t="n">
         <v>0</v>
       </c>
+      <c r="W364" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="365">
       <c r="A365" t="n">
@@ -25279,6 +26373,9 @@
       <c r="V365" t="n">
         <v>0</v>
       </c>
+      <c r="W365" t="n">
+        <v>5.4</v>
+      </c>
     </row>
     <row r="366">
       <c r="A366" t="n">
@@ -25347,6 +26444,9 @@
       <c r="V366" t="n">
         <v>0</v>
       </c>
+      <c r="W366" t="n">
+        <v>7.9</v>
+      </c>
     </row>
     <row r="367">
       <c r="A367" t="n">
@@ -25415,6 +26515,9 @@
       <c r="V367" t="n">
         <v>0</v>
       </c>
+      <c r="W367" t="n">
+        <v>12.8</v>
+      </c>
     </row>
     <row r="368">
       <c r="A368" t="n">
@@ -25483,6 +26586,9 @@
       <c r="V368" t="n">
         <v>1</v>
       </c>
+      <c r="W368" t="n">
+        <v>31.6</v>
+      </c>
     </row>
     <row r="369">
       <c r="A369" t="n">
@@ -25551,6 +26657,9 @@
       <c r="V369" t="n">
         <v>0</v>
       </c>
+      <c r="W369" t="n">
+        <v>18.4</v>
+      </c>
     </row>
     <row r="370">
       <c r="A370" t="n">
@@ -25619,6 +26728,9 @@
       <c r="V370" t="n">
         <v>0</v>
       </c>
+      <c r="W370" t="n">
+        <v>30.1</v>
+      </c>
     </row>
     <row r="371">
       <c r="A371" t="n">
@@ -25687,6 +26799,9 @@
       <c r="V371" t="n">
         <v>1</v>
       </c>
+      <c r="W371" t="n">
+        <v>19.8</v>
+      </c>
     </row>
     <row r="372">
       <c r="A372" t="n">
@@ -25755,6 +26870,9 @@
       <c r="V372" t="n">
         <v>1</v>
       </c>
+      <c r="W372" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="373">
       <c r="A373" t="n">
@@ -25823,6 +26941,9 @@
       <c r="V373" t="n">
         <v>1</v>
       </c>
+      <c r="W373" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="374">
       <c r="A374" t="n">
@@ -25891,6 +27012,9 @@
       <c r="V374" t="n">
         <v>0</v>
       </c>
+      <c r="W374" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="375">
       <c r="A375" t="n">
@@ -25959,6 +27083,9 @@
       <c r="V375" t="n">
         <v>0</v>
       </c>
+      <c r="W375" t="n">
+        <v>24.2</v>
+      </c>
     </row>
     <row r="376">
       <c r="A376" t="n">
@@ -26027,6 +27154,9 @@
       <c r="V376" t="n">
         <v>0</v>
       </c>
+      <c r="W376" t="n">
+        <v>16.9</v>
+      </c>
     </row>
     <row r="377">
       <c r="A377" t="n">
@@ -26095,6 +27225,9 @@
       <c r="V377" t="n">
         <v>0</v>
       </c>
+      <c r="W377" t="n">
+        <v>26.6</v>
+      </c>
     </row>
     <row r="378">
       <c r="A378" t="n">
@@ -26163,6 +27296,9 @@
       <c r="V378" t="n">
         <v>0</v>
       </c>
+      <c r="W378" t="n">
+        <v>19.7</v>
+      </c>
     </row>
     <row r="379">
       <c r="A379" t="n">
@@ -26231,6 +27367,9 @@
       <c r="V379" t="n">
         <v>0</v>
       </c>
+      <c r="W379" t="n">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="380">
       <c r="A380" t="n">
@@ -26299,6 +27438,9 @@
       <c r="V380" t="n">
         <v>0</v>
       </c>
+      <c r="W380" t="n">
+        <v>32.2</v>
+      </c>
     </row>
     <row r="381">
       <c r="A381" t="n">
@@ -26367,6 +27509,9 @@
       <c r="V381" t="n">
         <v>0</v>
       </c>
+      <c r="W381" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="382">
       <c r="A382" t="n">
@@ -26435,6 +27580,9 @@
       <c r="V382" t="n">
         <v>1</v>
       </c>
+      <c r="W382" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="383">
       <c r="A383" t="n">
@@ -26503,6 +27651,9 @@
       <c r="V383" t="n">
         <v>1</v>
       </c>
+      <c r="W383" t="n">
+        <v>29.1</v>
+      </c>
     </row>
     <row r="384">
       <c r="A384" t="n">
@@ -26571,6 +27722,9 @@
       <c r="V384" t="n">
         <v>0</v>
       </c>
+      <c r="W384" t="n">
+        <v>34.7</v>
+      </c>
     </row>
     <row r="385">
       <c r="A385" t="n">
@@ -26639,6 +27793,9 @@
       <c r="V385" t="n">
         <v>0</v>
       </c>
+      <c r="W385" t="n">
+        <v>13.4</v>
+      </c>
     </row>
     <row r="386">
       <c r="A386" t="n">
@@ -26707,6 +27864,9 @@
       <c r="V386" t="n">
         <v>0</v>
       </c>
+      <c r="W386" t="n">
+        <v>10.7</v>
+      </c>
     </row>
     <row r="387">
       <c r="A387" t="n">
@@ -26775,6 +27935,9 @@
       <c r="V387" t="n">
         <v>1</v>
       </c>
+      <c r="W387" t="n">
+        <v>31.1</v>
+      </c>
     </row>
     <row r="388">
       <c r="A388" t="n">
@@ -26843,6 +28006,9 @@
       <c r="V388" t="n">
         <v>0</v>
       </c>
+      <c r="W388" t="n">
+        <v>26.1</v>
+      </c>
     </row>
     <row r="389">
       <c r="A389" t="n">
@@ -26911,6 +28077,9 @@
       <c r="V389" t="n">
         <v>0</v>
       </c>
+      <c r="W389" t="n">
+        <v>19.4</v>
+      </c>
     </row>
     <row r="390">
       <c r="A390" t="n">
@@ -26979,6 +28148,9 @@
       <c r="V390" t="n">
         <v>0</v>
       </c>
+      <c r="W390" t="n">
+        <v>21.2</v>
+      </c>
     </row>
     <row r="391">
       <c r="A391" t="n">
@@ -27047,6 +28219,9 @@
       <c r="V391" t="n">
         <v>0</v>
       </c>
+      <c r="W391" t="n">
+        <v>36.8</v>
+      </c>
     </row>
     <row r="392">
       <c r="A392" t="n">
@@ -27115,6 +28290,9 @@
       <c r="V392" t="n">
         <v>1</v>
       </c>
+      <c r="W392" t="n">
+        <v>17.1</v>
+      </c>
     </row>
     <row r="393">
       <c r="A393" t="n">
@@ -27183,6 +28361,9 @@
       <c r="V393" t="n">
         <v>0</v>
       </c>
+      <c r="W393" t="n">
+        <v>33.7</v>
+      </c>
     </row>
     <row r="394">
       <c r="A394" t="n">
@@ -27251,6 +28432,9 @@
       <c r="V394" t="n">
         <v>0</v>
       </c>
+      <c r="W394" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="395">
       <c r="A395" t="n">
@@ -27319,6 +28503,9 @@
       <c r="V395" t="n">
         <v>1</v>
       </c>
+      <c r="W395" t="n">
+        <v>13.7</v>
+      </c>
     </row>
     <row r="396">
       <c r="A396" t="n">
@@ -27387,6 +28574,9 @@
       <c r="V396" t="n">
         <v>0</v>
       </c>
+      <c r="W396" t="n">
+        <v>24.5</v>
+      </c>
     </row>
     <row r="397">
       <c r="A397" t="n">
@@ -27455,6 +28645,9 @@
       <c r="V397" t="n">
         <v>1</v>
       </c>
+      <c r="W397" t="n">
+        <v>15.1</v>
+      </c>
     </row>
     <row r="398">
       <c r="A398" t="n">
@@ -27523,6 +28716,9 @@
       <c r="V398" t="n">
         <v>0</v>
       </c>
+      <c r="W398" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="399">
       <c r="A399" t="n">
@@ -27591,6 +28787,9 @@
       <c r="V399" t="n">
         <v>0</v>
       </c>
+      <c r="W399" t="n">
+        <v>7.7</v>
+      </c>
     </row>
     <row r="400">
       <c r="A400" t="n">
@@ -27659,6 +28858,9 @@
       <c r="V400" t="n">
         <v>0</v>
       </c>
+      <c r="W400" t="n">
+        <v>37.2</v>
+      </c>
     </row>
     <row r="401">
       <c r="A401" t="n">
@@ -27727,6 +28929,9 @@
       <c r="V401" t="n">
         <v>0</v>
       </c>
+      <c r="W401" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="402">
       <c r="A402" t="n">
@@ -27795,6 +29000,9 @@
       <c r="V402" t="n">
         <v>0</v>
       </c>
+      <c r="W402" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="403">
       <c r="A403" t="n">
@@ -27863,6 +29071,9 @@
       <c r="V403" t="n">
         <v>1</v>
       </c>
+      <c r="W403" t="n">
+        <v>11.5</v>
+      </c>
     </row>
     <row r="404">
       <c r="A404" t="n">
@@ -27931,6 +29142,9 @@
       <c r="V404" t="n">
         <v>0</v>
       </c>
+      <c r="W404" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="405">
       <c r="A405" t="n">
@@ -27999,6 +29213,9 @@
       <c r="V405" t="n">
         <v>1</v>
       </c>
+      <c r="W405" t="n">
+        <v>28.2</v>
+      </c>
     </row>
     <row r="406">
       <c r="A406" t="n">
@@ -28067,6 +29284,9 @@
       <c r="V406" t="n">
         <v>0</v>
       </c>
+      <c r="W406" t="n">
+        <v>45.5</v>
+      </c>
     </row>
     <row r="407">
       <c r="A407" t="n">
@@ -28135,6 +29355,9 @@
       <c r="V407" t="n">
         <v>0</v>
       </c>
+      <c r="W407" t="n">
+        <v>24.7</v>
+      </c>
     </row>
     <row r="408">
       <c r="A408" t="n">
@@ -28203,6 +29426,9 @@
       <c r="V408" t="n">
         <v>0</v>
       </c>
+      <c r="W408" t="n">
+        <v>7.6</v>
+      </c>
     </row>
     <row r="409">
       <c r="A409" t="n">
@@ -28271,6 +29497,9 @@
       <c r="V409" t="n">
         <v>1</v>
       </c>
+      <c r="W409" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="410">
       <c r="A410" t="n">
@@ -28339,6 +29568,9 @@
       <c r="V410" t="n">
         <v>1</v>
       </c>
+      <c r="W410" t="n">
+        <v>35.8</v>
+      </c>
     </row>
     <row r="411">
       <c r="A411" t="n">
@@ -28407,6 +29639,9 @@
       <c r="V411" t="n">
         <v>0</v>
       </c>
+      <c r="W411" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="412">
       <c r="A412" t="n">
@@ -28475,6 +29710,9 @@
       <c r="V412" t="n">
         <v>0</v>
       </c>
+      <c r="W412" t="n">
+        <v>36.5</v>
+      </c>
     </row>
     <row r="413">
       <c r="A413" t="n">
@@ -28543,6 +29781,9 @@
       <c r="V413" t="n">
         <v>0</v>
       </c>
+      <c r="W413" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="414">
       <c r="A414" t="n">
@@ -28611,6 +29852,9 @@
       <c r="V414" t="n">
         <v>0</v>
       </c>
+      <c r="W414" t="n">
+        <v>31.1</v>
+      </c>
     </row>
     <row r="415">
       <c r="A415" t="n">
@@ -28679,6 +29923,9 @@
       <c r="V415" t="n">
         <v>0</v>
       </c>
+      <c r="W415" t="n">
+        <v>17.4</v>
+      </c>
     </row>
     <row r="416">
       <c r="A416" t="n">
@@ -28747,6 +29994,9 @@
       <c r="V416" t="n">
         <v>0</v>
       </c>
+      <c r="W416" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="417">
       <c r="A417" t="n">
@@ -28815,6 +30065,9 @@
       <c r="V417" t="n">
         <v>0</v>
       </c>
+      <c r="W417" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="418">
       <c r="A418" t="n">
@@ -28883,6 +30136,9 @@
       <c r="V418" t="n">
         <v>0</v>
       </c>
+      <c r="W418" t="n">
+        <v>28.3</v>
+      </c>
     </row>
     <row r="419">
       <c r="A419" t="n">
@@ -28951,6 +30207,9 @@
       <c r="V419" t="n">
         <v>0</v>
       </c>
+      <c r="W419" t="n">
+        <v>34.3</v>
+      </c>
     </row>
     <row r="420">
       <c r="A420" t="n">
@@ -29019,6 +30278,9 @@
       <c r="V420" t="n">
         <v>0</v>
       </c>
+      <c r="W420" t="n">
+        <v>19.5</v>
+      </c>
     </row>
     <row r="421">
       <c r="A421" t="n">
@@ -29087,6 +30349,9 @@
       <c r="V421" t="n">
         <v>0</v>
       </c>
+      <c r="W421" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="422">
       <c r="A422" t="n">
@@ -29155,6 +30420,9 @@
       <c r="V422" t="n">
         <v>0</v>
       </c>
+      <c r="W422" t="n">
+        <v>31</v>
+      </c>
     </row>
     <row r="423">
       <c r="A423" t="n">
@@ -29223,6 +30491,9 @@
       <c r="V423" t="n">
         <v>0</v>
       </c>
+      <c r="W423" t="n">
+        <v>39.6</v>
+      </c>
     </row>
     <row r="424">
       <c r="A424" t="n">
@@ -29291,6 +30562,9 @@
       <c r="V424" t="n">
         <v>0</v>
       </c>
+      <c r="W424" t="n">
+        <v>24.3</v>
+      </c>
     </row>
     <row r="425">
       <c r="A425" t="n">
@@ -29359,6 +30633,9 @@
       <c r="V425" t="n">
         <v>0</v>
       </c>
+      <c r="W425" t="n">
+        <v>0.9</v>
+      </c>
     </row>
     <row r="426">
       <c r="A426" t="n">
@@ -29427,6 +30704,9 @@
       <c r="V426" t="n">
         <v>0</v>
       </c>
+      <c r="W426" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="427">
       <c r="A427" t="n">
@@ -29495,6 +30775,9 @@
       <c r="V427" t="n">
         <v>1</v>
       </c>
+      <c r="W427" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="428">
       <c r="A428" t="n">
@@ -29563,6 +30846,9 @@
       <c r="V428" t="n">
         <v>1</v>
       </c>
+      <c r="W428" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="429">
       <c r="A429" t="n">
@@ -29631,6 +30917,9 @@
       <c r="V429" t="n">
         <v>1</v>
       </c>
+      <c r="W429" t="n">
+        <v>37.2</v>
+      </c>
     </row>
     <row r="430">
       <c r="A430" t="n">
@@ -29699,6 +30988,9 @@
       <c r="V430" t="n">
         <v>0</v>
       </c>
+      <c r="W430" t="n">
+        <v>15.7</v>
+      </c>
     </row>
     <row r="431">
       <c r="A431" t="n">
@@ -29767,6 +31059,9 @@
       <c r="V431" t="n">
         <v>1</v>
       </c>
+      <c r="W431" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="432">
       <c r="A432" t="n">
@@ -29835,6 +31130,9 @@
       <c r="V432" t="n">
         <v>0</v>
       </c>
+      <c r="W432" t="n">
+        <v>19.2</v>
+      </c>
     </row>
     <row r="433">
       <c r="A433" t="n">
@@ -29903,6 +31201,9 @@
       <c r="V433" t="n">
         <v>0</v>
       </c>
+      <c r="W433" t="n">
+        <v>29.6</v>
+      </c>
     </row>
     <row r="434">
       <c r="A434" t="n">
@@ -29971,6 +31272,9 @@
       <c r="V434" t="n">
         <v>0</v>
       </c>
+      <c r="W434" t="n">
+        <v>29.1</v>
+      </c>
     </row>
     <row r="435">
       <c r="A435" t="n">
@@ -30039,6 +31343,9 @@
       <c r="V435" t="n">
         <v>0</v>
       </c>
+      <c r="W435" t="n">
+        <v>39.3</v>
+      </c>
     </row>
     <row r="436">
       <c r="A436" t="n">
@@ -30107,6 +31414,9 @@
       <c r="V436" t="n">
         <v>0</v>
       </c>
+      <c r="W436" t="n">
+        <v>29.3</v>
+      </c>
     </row>
     <row r="437">
       <c r="A437" t="n">
@@ -30175,6 +31485,9 @@
       <c r="V437" t="n">
         <v>0</v>
       </c>
+      <c r="W437" t="n">
+        <v>15.8</v>
+      </c>
     </row>
     <row r="438">
       <c r="A438" t="n">
@@ -30243,6 +31556,9 @@
       <c r="V438" t="n">
         <v>0</v>
       </c>
+      <c r="W438" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="439">
       <c r="A439" t="n">
@@ -30311,6 +31627,9 @@
       <c r="V439" t="n">
         <v>0</v>
       </c>
+      <c r="W439" t="n">
+        <v>26.6</v>
+      </c>
     </row>
     <row r="440">
       <c r="A440" t="n">
@@ -30379,6 +31698,9 @@
       <c r="V440" t="n">
         <v>0</v>
       </c>
+      <c r="W440" t="n">
+        <v>28.3</v>
+      </c>
     </row>
     <row r="441">
       <c r="A441" t="n">
@@ -30447,6 +31769,9 @@
       <c r="V441" t="n">
         <v>0</v>
       </c>
+      <c r="W441" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="442">
       <c r="A442" t="n">
@@ -30515,6 +31840,9 @@
       <c r="V442" t="n">
         <v>0</v>
       </c>
+      <c r="W442" t="n">
+        <v>36.9</v>
+      </c>
     </row>
     <row r="443">
       <c r="A443" t="n">
@@ -30583,6 +31911,9 @@
       <c r="V443" t="n">
         <v>1</v>
       </c>
+      <c r="W443" t="n">
+        <v>15.3</v>
+      </c>
     </row>
     <row r="444">
       <c r="A444" t="n">
@@ -30651,6 +31982,9 @@
       <c r="V444" t="n">
         <v>0</v>
       </c>
+      <c r="W444" t="n">
+        <v>31.5</v>
+      </c>
     </row>
     <row r="445">
       <c r="A445" t="n">
@@ -30719,6 +32053,9 @@
       <c r="V445" t="n">
         <v>0</v>
       </c>
+      <c r="W445" t="n">
+        <v>11.9</v>
+      </c>
     </row>
     <row r="446">
       <c r="A446" t="n">
@@ -30787,6 +32124,9 @@
       <c r="V446" t="n">
         <v>0</v>
       </c>
+      <c r="W446" t="n">
+        <v>27.4</v>
+      </c>
     </row>
     <row r="447">
       <c r="A447" t="n">
@@ -30855,6 +32195,9 @@
       <c r="V447" t="n">
         <v>0</v>
       </c>
+      <c r="W447" t="n">
+        <v>38.1</v>
+      </c>
     </row>
     <row r="448">
       <c r="A448" t="n">
@@ -30923,6 +32266,9 @@
       <c r="V448" t="n">
         <v>0</v>
       </c>
+      <c r="W448" t="n">
+        <v>26.2</v>
+      </c>
     </row>
     <row r="449">
       <c r="A449" t="n">
@@ -30991,6 +32337,9 @@
       <c r="V449" t="n">
         <v>0</v>
       </c>
+      <c r="W449" t="n">
+        <v>30.4</v>
+      </c>
     </row>
     <row r="450">
       <c r="A450" t="n">
@@ -31059,6 +32408,9 @@
       <c r="V450" t="n">
         <v>0</v>
       </c>
+      <c r="W450" t="n">
+        <v>31.2</v>
+      </c>
     </row>
     <row r="451">
       <c r="A451" t="n">
@@ -31127,6 +32479,9 @@
       <c r="V451" t="n">
         <v>0</v>
       </c>
+      <c r="W451" t="n">
+        <v>19.4</v>
+      </c>
     </row>
     <row r="452">
       <c r="A452" t="n">
@@ -31195,6 +32550,9 @@
       <c r="V452" t="n">
         <v>0</v>
       </c>
+      <c r="W452" t="n">
+        <v>27.5</v>
+      </c>
     </row>
     <row r="453">
       <c r="A453" t="n">
@@ -31263,6 +32621,9 @@
       <c r="V453" t="n">
         <v>0</v>
       </c>
+      <c r="W453" t="n">
+        <v>13.3</v>
+      </c>
     </row>
     <row r="454">
       <c r="A454" t="n">
@@ -31331,6 +32692,9 @@
       <c r="V454" t="n">
         <v>0</v>
       </c>
+      <c r="W454" t="n">
+        <v>20.3</v>
+      </c>
     </row>
     <row r="455">
       <c r="A455" t="n">
@@ -31399,6 +32763,9 @@
       <c r="V455" t="n">
         <v>0</v>
       </c>
+      <c r="W455" t="n">
+        <v>39.3</v>
+      </c>
     </row>
     <row r="456">
       <c r="A456" t="n">
@@ -31467,6 +32834,9 @@
       <c r="V456" t="n">
         <v>0</v>
       </c>
+      <c r="W456" t="n">
+        <v>26.6</v>
+      </c>
     </row>
     <row r="457">
       <c r="A457" t="n">
@@ -31535,6 +32905,9 @@
       <c r="V457" t="n">
         <v>0</v>
       </c>
+      <c r="W457" t="n">
+        <v>31.7</v>
+      </c>
     </row>
     <row r="458">
       <c r="A458" t="n">
@@ -31603,6 +32976,9 @@
       <c r="V458" t="n">
         <v>0</v>
       </c>
+      <c r="W458" t="n">
+        <v>9.1</v>
+      </c>
     </row>
     <row r="459">
       <c r="A459" t="n">
@@ -31671,6 +33047,9 @@
       <c r="V459" t="n">
         <v>0</v>
       </c>
+      <c r="W459" t="n">
+        <v>16.2</v>
+      </c>
     </row>
     <row r="460">
       <c r="A460" t="n">
@@ -31739,6 +33118,9 @@
       <c r="V460" t="n">
         <v>0</v>
       </c>
+      <c r="W460" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="461">
       <c r="A461" t="n">
@@ -31807,6 +33189,9 @@
       <c r="V461" t="n">
         <v>0</v>
       </c>
+      <c r="W461" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="462">
       <c r="A462" t="n">
@@ -31875,6 +33260,9 @@
       <c r="V462" t="n">
         <v>1</v>
       </c>
+      <c r="W462" t="n">
+        <v>27.9</v>
+      </c>
     </row>
     <row r="463">
       <c r="A463" t="n">
@@ -31943,6 +33331,9 @@
       <c r="V463" t="n">
         <v>1</v>
       </c>
+      <c r="W463" t="n">
+        <v>29.3</v>
+      </c>
     </row>
     <row r="464">
       <c r="A464" t="n">
@@ -32011,6 +33402,9 @@
       <c r="V464" t="n">
         <v>0</v>
       </c>
+      <c r="W464" t="n">
+        <v>35.7</v>
+      </c>
     </row>
     <row r="465">
       <c r="A465" t="n">
@@ -32079,6 +33473,9 @@
       <c r="V465" t="n">
         <v>0</v>
       </c>
+      <c r="W465" t="n">
+        <v>17.7</v>
+      </c>
     </row>
     <row r="466">
       <c r="A466" t="n">
@@ -32147,6 +33544,9 @@
       <c r="V466" t="n">
         <v>0</v>
       </c>
+      <c r="W466" t="n">
+        <v>50.3</v>
+      </c>
     </row>
     <row r="467">
       <c r="A467" t="n">
@@ -32215,6 +33615,9 @@
       <c r="V467" t="n">
         <v>0</v>
       </c>
+      <c r="W467" t="n">
+        <v>9.4</v>
+      </c>
     </row>
     <row r="468">
       <c r="A468" t="n">
@@ -32283,6 +33686,9 @@
       <c r="V468" t="n">
         <v>0</v>
       </c>
+      <c r="W468" t="n">
+        <v>14.6</v>
+      </c>
     </row>
     <row r="469">
       <c r="A469" t="n">
@@ -32350,6 +33756,9 @@
       </c>
       <c r="V469" t="n">
         <v>0</v>
+      </c>
+      <c r="W469" t="n">
+        <v>16.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>